<commit_message>
Edited description of project, and after verifying all papers are included, I realized that my raw data had two papers that were being ecluded due to notes I had within those cells (D*, D and E), so I edited those to be consisten with the others (to D and E, respectively), while moving the notes to cells in G. Saved fig 5, even though I don't feel it is particularly helpful.
</commit_message>
<xml_diff>
--- a/data/raw/coded_most_recent_vulgaris.xlsx
+++ b/data/raw/coded_most_recent_vulgaris.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://miamiedu-my.sharepoint.com/personal/jxk1462_miami_edu/Documents/Desktop/EVR628/GitHub Portfolio/portfolio/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="8_{47C56A75-2044-4A33-9E23-147D2FC85DA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CA3E1686-E2D8-41AF-9414-06F7739A9B6F}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="8_{47C56A75-2044-4A33-9E23-147D2FC85DA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{210993FC-1865-402C-9771-D75AB57CC2E2}"/>
   <bookViews>
-    <workbookView xWindow="2220" yWindow="1815" windowWidth="23010" windowHeight="11970" activeTab="1" xr2:uid="{D58EA8E2-D2B4-4047-B1D6-8B88B0BE0854}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="1" xr2:uid="{D58EA8E2-D2B4-4047-B1D6-8B88B0BE0854}"/>
   </bookViews>
   <sheets>
     <sheet name="savedrecs" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7165" uniqueCount="4175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7167" uniqueCount="4177">
   <si>
     <t>Authors</t>
   </si>
@@ -15371,6 +15371,12 @@
   </si>
   <si>
     <t>Wales, England</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>E</t>
   </si>
 </sst>
 </file>
@@ -23209,7 +23215,7 @@
       <c r="AP54" s="4" t="s">
         <v>3651</v>
       </c>
-      <c r="AQ54" t="s">
+      <c r="AQ54" s="4" t="s">
         <v>3917</v>
       </c>
       <c r="AR54">
@@ -42994,7 +43000,7 @@
         <v>3633</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A49" s="4" t="s">
         <v>3637</v>
       </c>
@@ -43014,7 +43020,7 @@
         <v>3633</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A50" s="4" t="s">
         <v>3667</v>
       </c>
@@ -43034,7 +43040,7 @@
         <v>3708</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A51" s="4" t="s">
         <v>3684</v>
       </c>
@@ -43054,7 +43060,7 @@
         <v>3653</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A52" s="4" t="s">
         <v>3656</v>
       </c>
@@ -43074,7 +43080,7 @@
         <v>3653</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A53" s="4" t="s">
         <v>3656</v>
       </c>
@@ -43094,7 +43100,7 @@
         <v>3633</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A54" s="4" t="s">
         <v>3658</v>
       </c>
@@ -43111,10 +43117,13 @@
         <v>3651</v>
       </c>
       <c r="F54" s="4" t="s">
-        <v>3918</v>
+        <v>3653</v>
+      </c>
+      <c r="G54" s="4" t="s">
+        <v>4175</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A55" s="4" t="s">
         <v>3694</v>
       </c>
@@ -43134,7 +43143,7 @@
         <v>3653</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A56" s="4" t="s">
         <v>3684</v>
       </c>
@@ -43154,7 +43163,7 @@
         <v>3653</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>3684</v>
       </c>
@@ -43174,7 +43183,7 @@
         <v>3653</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>3684</v>
       </c>
@@ -43194,7 +43203,7 @@
         <v>3633</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>3656</v>
       </c>
@@ -43214,7 +43223,7 @@
         <v>3708</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>3694</v>
       </c>
@@ -43234,7 +43243,7 @@
         <v>3653</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A61" s="4" t="s">
         <v>3658</v>
       </c>
@@ -43254,7 +43263,7 @@
         <v>3633</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>3667</v>
       </c>
@@ -43274,7 +43283,7 @@
         <v>3708</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>3876</v>
       </c>
@@ -43294,7 +43303,7 @@
         <v>3963</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>3657</v>
       </c>
@@ -43634,7 +43643,7 @@
         <v>3653</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A81" s="4" t="s">
         <v>3647</v>
       </c>
@@ -43654,7 +43663,7 @@
         <v>3653</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A82" s="4" t="s">
         <v>3637</v>
       </c>
@@ -43674,7 +43683,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A83" s="4" t="s">
         <v>3637</v>
       </c>
@@ -43694,7 +43703,7 @@
         <v>3633</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A84" s="4" t="s">
         <v>3647</v>
       </c>
@@ -43711,10 +43720,13 @@
         <v>3706</v>
       </c>
       <c r="F84" s="4" t="s">
+        <v>4176</v>
+      </c>
+      <c r="G84" s="4" t="s">
         <v>4073</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A85" s="4" t="s">
         <v>3637</v>
       </c>
@@ -43734,7 +43746,7 @@
         <v>3633</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A86" s="4" t="s">
         <v>3876</v>
       </c>
@@ -43754,7 +43766,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A87" s="4" t="s">
         <v>3684</v>
       </c>
@@ -43774,7 +43786,7 @@
         <v>3653</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A88" s="4" t="s">
         <v>3657</v>
       </c>
@@ -43794,7 +43806,7 @@
         <v>3653</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A89" s="4" t="s">
         <v>3637</v>
       </c>
@@ -43814,7 +43826,7 @@
         <v>3633</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A90" s="4" t="s">
         <v>3679</v>
       </c>
@@ -43834,7 +43846,7 @@
         <v>3653</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A91" s="4" t="s">
         <v>3637</v>
       </c>
@@ -43854,7 +43866,7 @@
         <v>3633</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A92" s="4" t="s">
         <v>3637</v>
       </c>
@@ -43874,7 +43886,7 @@
         <v>3633</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A93" s="4" t="s">
         <v>3876</v>
       </c>
@@ -43894,7 +43906,7 @@
         <v>3653</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A94" s="4" t="s">
         <v>3656</v>
       </c>
@@ -43914,7 +43926,7 @@
         <v>3653</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A95" s="4" t="s">
         <v>3684</v>
       </c>
@@ -43934,7 +43946,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A96" s="4" t="s">
         <v>3798</v>
       </c>

</xml_diff>